<commit_message>
Atualização 29/10 - 30/10
</commit_message>
<xml_diff>
--- a/painel-de-saldos.xlsx
+++ b/painel-de-saldos.xlsx
@@ -411,7 +411,7 @@
         <v/>
       </c>
       <c r="B2" t="str">
-        <v>Painel de Saldos Diários 28/10 à 29/10/2026</v>
+        <v>Painel de Saldos Diários 29/10 à 30/10/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Master Educação Profissional</v>
@@ -433,7 +433,7 @@
         <v xml:space="preserve">Saldo Anterior ( A ) </v>
       </c>
       <c r="C4">
-        <v>41941.41</v>
+        <v>63479.39</v>
       </c>
     </row>
     <row r="5">
@@ -444,7 +444,7 @@
         <v xml:space="preserve">Entrada  ( B ) </v>
       </c>
       <c r="C5">
-        <v>283.83</v>
+        <v>485.38</v>
       </c>
     </row>
     <row r="6">
@@ -455,7 +455,7 @@
         <v xml:space="preserve">Saída ( C ) </v>
       </c>
       <c r="C6">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -466,7 +466,7 @@
         <v xml:space="preserve">Saldo Atual ( A + B - C ) </v>
       </c>
       <c r="C7">
-        <v>41225.240000000005</v>
+        <v>63964.77</v>
       </c>
     </row>
     <row r="8">
@@ -485,7 +485,7 @@
         <v xml:space="preserve">Saldo Anterior ( A ) </v>
       </c>
       <c r="C9">
-        <v>-676.05</v>
+        <v>-1776.16</v>
       </c>
     </row>
     <row r="10">
@@ -496,7 +496,7 @@
         <v xml:space="preserve">Entrada  ( B ) </v>
       </c>
       <c r="C10">
-        <v>1265.5</v>
+        <v>805.11</v>
       </c>
     </row>
     <row r="11">
@@ -507,7 +507,7 @@
         <v xml:space="preserve">Saída ( C ) </v>
       </c>
       <c r="C11">
-        <v>1.93</v>
+        <v>25.09</v>
       </c>
     </row>
     <row r="12">
@@ -518,7 +518,7 @@
         <v xml:space="preserve">Saldo Atual ( A + B - C ) </v>
       </c>
       <c r="C12">
-        <v>587.5200000000001</v>
+        <v>-996.1400000000001</v>
       </c>
     </row>
     <row r="13">
@@ -589,7 +589,7 @@
         <v xml:space="preserve">Saldo Anterior ( A ) </v>
       </c>
       <c r="C19">
-        <v>273.06</v>
+        <v>273.18</v>
       </c>
     </row>
     <row r="20">
@@ -622,7 +622,7 @@
         <v xml:space="preserve">Saldo Atual da Conta de Aplicação </v>
       </c>
       <c r="C22">
-        <v>273.06</v>
+        <v>273.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>